<commit_message>
Add 4 missing flavors to Excel template
PISTACCHIO LARNAKA, NOCI UVETTA, FAVE FRESCHE & PECORINO,
STRAWBERRY FIELD FOREVER were computed by the extractor but
not found in the template → they appeared in orders but were
missing from the printed PDF.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gelato_flavors.xlsx
+++ b/gelato_flavors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29922"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC063E7A-B633-4349-A004-7438E8C824A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0817384A-A8AA-405D-9297-88747BB83D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="128">
   <si>
     <t>ALBICOCCA</t>
   </si>
@@ -121,9 +121,6 @@
     <t>NOCCIOLA</t>
   </si>
   <si>
-    <t>NOCI PECAN</t>
-  </si>
-  <si>
     <t>POLLICINA</t>
   </si>
   <si>
@@ -395,6 +392,18 @@
   </si>
   <si>
     <t>TOTAL:</t>
+  </si>
+  <si>
+    <t>P.LARNAKA</t>
+  </si>
+  <si>
+    <t>FAVE PECORINO</t>
+  </si>
+  <si>
+    <t>NOCI UVETTA</t>
+  </si>
+  <si>
+    <t>STRAWBERRY FILEDS</t>
   </si>
 </sst>
 </file>
@@ -483,11 +492,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -796,7 +805,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -812,593 +821,593 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="H1" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="6"/>
+        <v>71</v>
+      </c>
+      <c r="B2" s="5"/>
       <c r="C2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="6"/>
+      <c r="D2" s="5"/>
       <c r="E2" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F2" s="6"/>
+        <v>75</v>
+      </c>
+      <c r="F2" s="5"/>
       <c r="G2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="6"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="B3" s="5"/>
       <c r="C3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="6"/>
+      <c r="D3" s="5"/>
       <c r="E3" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="F3" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="F3" s="5"/>
       <c r="G3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="6"/>
+      <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="6"/>
+        <v>73</v>
+      </c>
+      <c r="B4" s="5"/>
       <c r="C4" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" s="6"/>
+        <v>91</v>
+      </c>
+      <c r="D4" s="5"/>
       <c r="E4" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" s="6"/>
+        <v>77</v>
+      </c>
+      <c r="F4" s="5"/>
       <c r="G4" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="H4" s="6"/>
+        <v>117</v>
+      </c>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="6"/>
+      <c r="B5" s="5"/>
       <c r="C5" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5" s="6"/>
+        <v>92</v>
+      </c>
+      <c r="D5" s="5"/>
       <c r="E5" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" s="6"/>
+        <v>78</v>
+      </c>
+      <c r="F5" s="5"/>
       <c r="G5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="6"/>
+      <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="6"/>
+        <v>44</v>
+      </c>
+      <c r="B6" s="5"/>
       <c r="C6" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="6"/>
+        <v>93</v>
+      </c>
+      <c r="D6" s="5"/>
       <c r="E6" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F6" s="6"/>
+        <v>79</v>
+      </c>
+      <c r="F6" s="5"/>
       <c r="G6" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="H6" s="6"/>
+        <v>109</v>
+      </c>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D7" s="6"/>
+        <v>95</v>
+      </c>
+      <c r="D7" s="5"/>
       <c r="E7" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F7" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="F7" s="5"/>
       <c r="G7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="6"/>
+      <c r="H7" s="5"/>
     </row>
     <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B8" s="6"/>
+        <v>94</v>
+      </c>
+      <c r="B8" s="5"/>
       <c r="C8" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D8" s="6"/>
+        <v>96</v>
+      </c>
+      <c r="D8" s="5"/>
       <c r="E8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F8" s="6"/>
+        <v>81</v>
+      </c>
+      <c r="F8" s="5"/>
       <c r="G8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H8" s="6"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="6"/>
+        <v>74</v>
+      </c>
+      <c r="B9" s="5"/>
       <c r="C9" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="6"/>
+        <v>108</v>
+      </c>
+      <c r="D9" s="5"/>
       <c r="E9" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" s="6"/>
+        <v>82</v>
+      </c>
+      <c r="F9" s="5"/>
       <c r="G9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="6"/>
+      <c r="H9" s="5"/>
     </row>
     <row r="10" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="6"/>
+        <v>125</v>
+      </c>
+      <c r="B10" s="5"/>
       <c r="C10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="6"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F10" s="6"/>
+        <v>83</v>
+      </c>
+      <c r="F10" s="5"/>
       <c r="G10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="6"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B11" s="6"/>
+        <v>25</v>
+      </c>
+      <c r="B11" s="5"/>
       <c r="C11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="6"/>
+        <v>43</v>
+      </c>
+      <c r="D11" s="5"/>
       <c r="E11" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F11" s="6"/>
+        <v>84</v>
+      </c>
+      <c r="F11" s="5"/>
       <c r="G11" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H11" s="6"/>
+        <v>110</v>
+      </c>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="6"/>
+        <v>107</v>
+      </c>
+      <c r="B12" s="5"/>
       <c r="C12" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="6"/>
+        <v>39</v>
+      </c>
+      <c r="D12" s="5"/>
       <c r="E12" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F12" s="6"/>
+        <v>85</v>
+      </c>
+      <c r="F12" s="5"/>
       <c r="G12" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="6"/>
+      <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="6"/>
+      <c r="B13" s="5"/>
       <c r="C13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="D13" s="5"/>
       <c r="E13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F13" s="6"/>
+        <v>86</v>
+      </c>
+      <c r="F13" s="5"/>
       <c r="G13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H13" s="6"/>
+      <c r="H13" s="5"/>
     </row>
     <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="6"/>
+        <v>89</v>
+      </c>
+      <c r="B14" s="5"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="6"/>
+      <c r="D14" s="5"/>
       <c r="E14" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="F14" s="6"/>
+        <v>87</v>
+      </c>
+      <c r="F14" s="5"/>
       <c r="G14" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="H14" s="6"/>
+        <v>114</v>
+      </c>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="6"/>
+        <v>27</v>
+      </c>
+      <c r="B15" s="5"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="6"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="F15" s="6"/>
+        <v>88</v>
+      </c>
+      <c r="F15" s="5"/>
       <c r="G15" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="H15" s="6"/>
+        <v>111</v>
+      </c>
+      <c r="H15" s="5"/>
     </row>
     <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="6"/>
+        <v>28</v>
+      </c>
+      <c r="B16" s="5"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="6"/>
+      <c r="D16" s="5"/>
       <c r="E16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="5"/>
       <c r="G16" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="H16" s="6"/>
+        <v>112</v>
+      </c>
+      <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="6"/>
+        <v>29</v>
+      </c>
+      <c r="B17" s="5"/>
       <c r="C17" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="6"/>
+        <v>53</v>
+      </c>
+      <c r="D17" s="5"/>
       <c r="E17" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F17" s="6"/>
+        <v>122</v>
+      </c>
+      <c r="F17" s="5"/>
       <c r="G17" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H17" s="6"/>
+      <c r="H17" s="5"/>
     </row>
     <row r="18" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="B18" s="5"/>
       <c r="C18" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="6"/>
+        <v>65</v>
+      </c>
+      <c r="D18" s="5"/>
       <c r="E18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="6"/>
+      <c r="F18" s="5"/>
       <c r="G18" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="6"/>
+      <c r="H18" s="5"/>
     </row>
     <row r="19" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" s="6"/>
+        <v>31</v>
+      </c>
+      <c r="B19" s="5"/>
       <c r="C19" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="D19" s="5"/>
       <c r="E19" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="F19" s="6"/>
+        <v>121</v>
+      </c>
+      <c r="F19" s="5"/>
       <c r="G19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H19" s="6"/>
+      <c r="H19" s="5"/>
     </row>
     <row r="20" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="6"/>
+        <v>52</v>
+      </c>
+      <c r="B20" s="5"/>
       <c r="C20" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="6"/>
+        <v>67</v>
+      </c>
+      <c r="D20" s="5"/>
       <c r="E20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F20" s="6"/>
+      <c r="F20" s="5"/>
       <c r="G20" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="H20" s="6"/>
+        <v>113</v>
+      </c>
+      <c r="H20" s="5"/>
     </row>
     <row r="21" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B21" s="6"/>
+        <v>32</v>
+      </c>
+      <c r="B21" s="5"/>
       <c r="C21" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="6"/>
+        <v>64</v>
+      </c>
+      <c r="D21" s="5"/>
       <c r="E21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="6"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H21" s="6"/>
+      <c r="H21" s="5"/>
     </row>
     <row r="22" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="6"/>
+        <v>97</v>
+      </c>
+      <c r="B22" s="5"/>
       <c r="C22" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D22" s="6"/>
+        <v>63</v>
+      </c>
+      <c r="D22" s="5"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H22" s="6"/>
+      <c r="H22" s="5"/>
     </row>
     <row r="23" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B23" s="6"/>
+        <v>126</v>
+      </c>
+      <c r="B23" s="5"/>
       <c r="C23" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="6"/>
+        <v>62</v>
+      </c>
+      <c r="D23" s="5"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H23" s="6"/>
+        <v>42</v>
+      </c>
+      <c r="H23" s="5"/>
     </row>
     <row r="24" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B24" s="6"/>
+        <v>98</v>
+      </c>
+      <c r="B24" s="5"/>
       <c r="C24" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="6"/>
+        <v>46</v>
+      </c>
+      <c r="D24" s="5"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="6"/>
+      <c r="H24" s="5"/>
     </row>
     <row r="25" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B25" s="6"/>
+        <v>99</v>
+      </c>
+      <c r="B25" s="5"/>
       <c r="C25" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="6"/>
+        <v>56</v>
+      </c>
+      <c r="D25" s="5"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="6"/>
+      <c r="H25" s="5"/>
     </row>
     <row r="26" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="6"/>
+        <v>124</v>
+      </c>
+      <c r="B26" s="5"/>
       <c r="C26" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" s="6"/>
+        <v>57</v>
+      </c>
+      <c r="D26" s="5"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H26" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="H26" s="5"/>
     </row>
     <row r="27" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="6"/>
+        <v>100</v>
+      </c>
+      <c r="B27" s="5"/>
       <c r="C27" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" s="6"/>
+        <v>58</v>
+      </c>
+      <c r="D27" s="5"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="H27" s="6"/>
+        <v>115</v>
+      </c>
+      <c r="H27" s="5"/>
     </row>
     <row r="28" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" s="6"/>
+        <v>33</v>
+      </c>
+      <c r="B28" s="5"/>
       <c r="C28" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" s="6"/>
+        <v>59</v>
+      </c>
+      <c r="D28" s="5"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H28" s="6"/>
+      <c r="H28" s="5"/>
     </row>
     <row r="29" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="6"/>
+        <v>35</v>
+      </c>
+      <c r="B29" s="5"/>
       <c r="C29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D29" s="6"/>
+        <v>54</v>
+      </c>
+      <c r="D29" s="5"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="H29" s="6"/>
+        <v>116</v>
+      </c>
+      <c r="H29" s="5"/>
     </row>
     <row r="30" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B30" s="6"/>
+        <v>101</v>
+      </c>
+      <c r="B30" s="5"/>
       <c r="C30" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D30" s="6"/>
+        <v>55</v>
+      </c>
+      <c r="D30" s="5"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="H30" s="6"/>
+        <v>118</v>
+      </c>
+      <c r="H30" s="5"/>
     </row>
     <row r="31" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B31" s="6"/>
+        <v>102</v>
+      </c>
+      <c r="B31" s="5"/>
       <c r="C31" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D31" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="D31" s="5"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="H31" s="6"/>
+        <v>69</v>
+      </c>
+      <c r="H31" s="5"/>
     </row>
     <row r="32" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="6"/>
+        <v>103</v>
+      </c>
+      <c r="B32" s="5"/>
       <c r="C32" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D32" s="6"/>
+        <v>61</v>
+      </c>
+      <c r="D32" s="5"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="H32" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="H32" s="5"/>
     </row>
     <row r="33" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="6"/>
+        <v>104</v>
+      </c>
+      <c r="B33" s="5"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="H33" s="6"/>
+        <v>119</v>
+      </c>
+      <c r="H33" s="5"/>
     </row>
     <row r="34" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B34" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="B34" s="5"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="H34" s="6"/>
+        <v>120</v>
+      </c>
+      <c r="H34" s="5"/>
     </row>
     <row r="35" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B35" s="6"/>
+        <v>37</v>
+      </c>
+      <c r="B35" s="5"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
@@ -1408,13 +1417,13 @@
     </row>
     <row r="36" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D36" s="5"/>
+        <v>105</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D36" s="6"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -1422,11 +1431,11 @@
     </row>
     <row r="37" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
+        <v>106</v>
+      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
@@ -1434,11 +1443,11 @@
     </row>
     <row r="38" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
+        <v>127</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -1446,15 +1455,30 @@
     </row>
     <row r="39" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B39" s="6"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
+        <v>38</v>
+      </c>
+      <c r="B39" s="5"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
+    </row>
+    <row r="40" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A40" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A41" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A42" s="4" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C18:C32">

</xml_diff>

<commit_message>
fix: add 4 missing flavors to PDF template (closes 5-unit gap)
BAKLAVA, PERA GORGONZOLA added to Gelato column.
FRAGOLE CHAMP, LIMONE & BASILICO added to Sorbetti column.
These were computed in orders (totalling 5 vaschette) but missing
from the template so they never appeared in the PDF.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gelato_flavors.xlsx
+++ b/gelato_flavors.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -837,6 +837,9 @@
       <c r="A35" t="str">
         <v>SEADAS</v>
       </c>
+      <c r="G35" t="str">
+        <v>FRAGOLE CHAMP</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -845,6 +848,9 @@
       <c r="C36" t="str">
         <v>TOTAL:</v>
       </c>
+      <c r="G36" t="str">
+        <v>LIMONE &amp; BASILICO</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -879,6 +885,16 @@
     <row r="46">
       <c r="A46" t="str">
         <v>NOCI PECAN</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>BAKLAVA</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>PERA GORGONZOLA</v>
       </c>
     </row>
   </sheetData>
@@ -887,7 +903,7 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: sync template names with SHOCAPP (closes 4-unit gap)
- C.BANANA → C. BANANA (spacing mismatch with SHOCAPP)
- Add COCCO AL RUM to Gelato column
- Add DRACARYS to Gelato column

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gelato_flavors.xlsx
+++ b/gelato_flavors.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H50"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -525,7 +525,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>C.BANANA</v>
+        <v>C. BANANA</v>
       </c>
       <c r="C9" t="str">
         <v>C. ZENZERO</v>
@@ -895,6 +895,16 @@
     <row r="48">
       <c r="A48" t="str">
         <v>PERA GORGONZOLA</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>COCCO AL RUM</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>DRACARYS</v>
       </c>
     </row>
   </sheetData>
@@ -903,7 +913,7 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>